<commit_message>
Fix lead management fields, categories, imports and secure exports
</commit_message>
<xml_diff>
--- a/public/sample-import/lead-contact-sample.xlsx
+++ b/public/sample-import/lead-contact-sample.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
-  <si>
-    <t>client_name</t>
-  </si>
-  <si>
-    <t>client_email</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>email</t>
   </si>
   <si>
     <t>mobile</t>
@@ -32,13 +32,10 @@
     <t>lead_requirements</t>
   </si>
   <si>
-    <t>company_name</t>
-  </si>
-  <si>
-    <t>Sample Lead</t>
-  </si>
-  <si>
-    <t>sample@example.com</t>
+    <t>Mohamed Ali</t>
+  </si>
+  <si>
+    <t>m.ali@example.com</t>
   </si>
   <si>
     <t>01110575930</t>
@@ -47,10 +44,31 @@
     <t>Umrah</t>
   </si>
   <si>
-    <t>Customer requests an Umrah package for two adults.</t>
-  </si>
-  <si>
-    <t>Sample Co</t>
+    <t>متطلبات الرحلة</t>
+  </si>
+  <si>
+    <t>Amina Hassan</t>
+  </si>
+  <si>
+    <t>amina.h@example.com</t>
+  </si>
+  <si>
+    <t>متطلبات العميل والخدمة المطلوبة</t>
+  </si>
+  <si>
+    <t>Omar Said</t>
+  </si>
+  <si>
+    <t>omar.said@example.com</t>
+  </si>
+  <si>
+    <t>01110000000</t>
+  </si>
+  <si>
+    <t>Hajj</t>
+  </si>
+  <si>
+    <t>Customer requires documentation</t>
   </si>
 </sst>
 </file>
@@ -390,10 +408,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -409,28 +427,56 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3">
+        <v>201110575930</v>
+      </c>
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>